<commit_message>
Session 20: 12 new engines (NEAR/SUI/APT/ARB + DOGE-H2/H3 + BNB-H2), updated roster xlsx, handoff
</commit_message>
<xml_diff>
--- a/chimera_engine_roster.xlsx
+++ b/chimera_engine_roster.xlsx
@@ -258,7 +258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -344,6 +344,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4795,264 +4802,236 @@
       <c r="S76" s="25" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="25" t="inlineStr">
-        <is>
-          <t>Profit Factor (PF)</t>
-        </is>
-      </c>
-      <c r="B77" s="25" t="n"/>
-      <c r="C77" s="25" t="n"/>
-      <c r="D77" s="25" t="n"/>
-      <c r="E77" s="25" t="n"/>
-      <c r="F77" s="25" t="n"/>
-      <c r="G77" s="25" t="n"/>
-      <c r="H77" s="25" t="n"/>
-      <c r="I77" s="25" t="n"/>
-      <c r="J77" s="25" t="n"/>
-      <c r="K77" s="25" t="n"/>
-      <c r="L77" s="25" t="n"/>
-      <c r="M77" s="25" t="n"/>
-      <c r="N77" s="25" t="n"/>
-      <c r="O77" s="25" t="n"/>
-      <c r="P77" s="25" t="n"/>
-      <c r="Q77" s="25" t="n"/>
+      <c r="A77" s="32" t="n"/>
+      <c r="B77" s="32" t="n"/>
+      <c r="C77" s="32" t="n"/>
+      <c r="D77" s="32" t="n"/>
+      <c r="E77" s="32" t="n"/>
+      <c r="F77" s="32" t="n"/>
+      <c r="G77" s="32" t="n"/>
+      <c r="H77" s="32" t="n"/>
+      <c r="I77" s="32" t="n"/>
+      <c r="J77" s="32" t="n"/>
+      <c r="K77" s="32" t="n"/>
+      <c r="L77" s="32" t="n"/>
+      <c r="M77" s="32" t="n"/>
+      <c r="N77" s="32" t="n"/>
+      <c r="O77" s="32" t="n"/>
+      <c r="P77" s="32" t="n"/>
+      <c r="Q77" s="32" t="n"/>
       <c r="R77" s="25" t="n"/>
       <c r="S77" s="25" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="28" t="inlineStr">
+      <c r="A78" s="43" t="inlineStr">
         <is>
           <t>SUMMARY: 49 TSMOM + 7 Tier-1 Counter-Trend + 5 Tier-2 Counter-Trend = 61 Total Engines (12 new in Session 20)</t>
         </is>
       </c>
-      <c r="B78" s="25" t="n"/>
-      <c r="C78" s="25" t="n"/>
-      <c r="D78" s="25" t="n"/>
-      <c r="E78" s="25" t="n"/>
-      <c r="F78" s="25" t="n"/>
-      <c r="G78" s="25" t="n"/>
-      <c r="H78" s="25" t="n"/>
-      <c r="I78" s="25" t="n"/>
-      <c r="J78" s="25" t="n"/>
-      <c r="K78" s="25" t="n"/>
-      <c r="L78" s="25" t="n"/>
-      <c r="M78" s="25" t="n"/>
-      <c r="N78" s="25" t="n"/>
-      <c r="O78" s="25" t="n"/>
-      <c r="P78" s="25" t="n"/>
-      <c r="Q78" s="25" t="n"/>
+      <c r="B78" s="32" t="n"/>
+      <c r="C78" s="32" t="n"/>
+      <c r="D78" s="32" t="n"/>
+      <c r="E78" s="32" t="n"/>
+      <c r="F78" s="32" t="n"/>
+      <c r="G78" s="32" t="n"/>
+      <c r="H78" s="32" t="n"/>
+      <c r="I78" s="32" t="n"/>
+      <c r="J78" s="32" t="n"/>
+      <c r="K78" s="32" t="n"/>
+      <c r="L78" s="32" t="n"/>
+      <c r="M78" s="32" t="n"/>
+      <c r="N78" s="32" t="n"/>
+      <c r="O78" s="32" t="n"/>
+      <c r="P78" s="32" t="n"/>
+      <c r="Q78" s="32" t="n"/>
       <c r="R78" s="25" t="n"/>
       <c r="S78" s="25" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="29" t="inlineStr">
-        <is>
-          <t>Anything above 1.0 is profitable; above 1.5 is strong; above 2.0 is excellent.</t>
-        </is>
-      </c>
-      <c r="B79" s="25" t="n"/>
-      <c r="C79" s="25" t="n"/>
-      <c r="D79" s="25" t="n"/>
-      <c r="E79" s="25" t="n"/>
-      <c r="F79" s="25" t="n"/>
-      <c r="G79" s="25" t="n"/>
-      <c r="H79" s="25" t="n"/>
-      <c r="I79" s="25" t="n"/>
-      <c r="J79" s="25" t="n"/>
-      <c r="K79" s="25" t="n"/>
-      <c r="L79" s="25" t="n"/>
-      <c r="M79" s="25" t="n"/>
-      <c r="N79" s="25" t="n"/>
-      <c r="O79" s="25" t="n"/>
-      <c r="P79" s="25" t="n"/>
-      <c r="Q79" s="25" t="n"/>
+      <c r="A79" s="44" t="n"/>
+      <c r="B79" s="32" t="n"/>
+      <c r="C79" s="32" t="n"/>
+      <c r="D79" s="32" t="n"/>
+      <c r="E79" s="32" t="n"/>
+      <c r="F79" s="32" t="n"/>
+      <c r="G79" s="32" t="n"/>
+      <c r="H79" s="32" t="n"/>
+      <c r="I79" s="32" t="n"/>
+      <c r="J79" s="32" t="n"/>
+      <c r="K79" s="32" t="n"/>
+      <c r="L79" s="32" t="n"/>
+      <c r="M79" s="32" t="n"/>
+      <c r="N79" s="32" t="n"/>
+      <c r="O79" s="32" t="n"/>
+      <c r="P79" s="32" t="n"/>
+      <c r="Q79" s="32" t="n"/>
       <c r="R79" s="25" t="n"/>
       <c r="S79" s="25" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="30" t="inlineStr">
+      <c r="A80" s="45" t="inlineStr">
         <is>
           <t>GRADE KEY:  STRONG = Nbr&gt;=90% &amp; PF&gt;=2.0 &amp; Trades&gt;=20  |  SOLID = Nbr&gt;=80% &amp; PF&gt;=1.5  |  GOOD = Nbr&gt;=60% &amp; PF&gt;=1.3  |  OK = Nbr&gt;=40% &amp; PF&gt;=1.15  |  WATCH = Below thresholds</t>
         </is>
       </c>
-      <c r="B80" s="25" t="n"/>
-      <c r="C80" s="25" t="n"/>
-      <c r="D80" s="25" t="n"/>
-      <c r="E80" s="25" t="n"/>
-      <c r="F80" s="25" t="n"/>
-      <c r="G80" s="25" t="n"/>
-      <c r="H80" s="25" t="n"/>
-      <c r="I80" s="25" t="n"/>
-      <c r="J80" s="25" t="n"/>
-      <c r="K80" s="25" t="n"/>
-      <c r="L80" s="25" t="n"/>
-      <c r="M80" s="25" t="n"/>
-      <c r="N80" s="25" t="n"/>
-      <c r="O80" s="25" t="n"/>
-      <c r="P80" s="25" t="n"/>
-      <c r="Q80" s="25" t="n"/>
+      <c r="B80" s="32" t="n"/>
+      <c r="C80" s="32" t="n"/>
+      <c r="D80" s="32" t="n"/>
+      <c r="E80" s="32" t="n"/>
+      <c r="F80" s="32" t="n"/>
+      <c r="G80" s="32" t="n"/>
+      <c r="H80" s="32" t="n"/>
+      <c r="I80" s="32" t="n"/>
+      <c r="J80" s="32" t="n"/>
+      <c r="K80" s="32" t="n"/>
+      <c r="L80" s="32" t="n"/>
+      <c r="M80" s="32" t="n"/>
+      <c r="N80" s="32" t="n"/>
+      <c r="O80" s="32" t="n"/>
+      <c r="P80" s="32" t="n"/>
+      <c r="Q80" s="32" t="n"/>
       <c r="R80" s="25" t="n"/>
       <c r="S80" s="25" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="25" t="inlineStr">
-        <is>
-          <t>Sharpe Ratio</t>
-        </is>
-      </c>
-      <c r="B81" s="25" t="n"/>
-      <c r="C81" s="25" t="n"/>
-      <c r="D81" s="25" t="n"/>
-      <c r="E81" s="25" t="n"/>
-      <c r="F81" s="25" t="n"/>
-      <c r="G81" s="25" t="n"/>
-      <c r="H81" s="25" t="n"/>
-      <c r="I81" s="25" t="n"/>
-      <c r="J81" s="25" t="n"/>
-      <c r="K81" s="25" t="n"/>
-      <c r="L81" s="25" t="n"/>
-      <c r="M81" s="25" t="n"/>
-      <c r="N81" s="25" t="n"/>
-      <c r="O81" s="25" t="n"/>
-      <c r="P81" s="25" t="n"/>
-      <c r="Q81" s="25" t="n"/>
+      <c r="A81" s="32" t="n"/>
+      <c r="B81" s="32" t="n"/>
+      <c r="C81" s="32" t="n"/>
+      <c r="D81" s="32" t="n"/>
+      <c r="E81" s="32" t="n"/>
+      <c r="F81" s="32" t="n"/>
+      <c r="G81" s="32" t="n"/>
+      <c r="H81" s="32" t="n"/>
+      <c r="I81" s="32" t="n"/>
+      <c r="J81" s="32" t="n"/>
+      <c r="K81" s="32" t="n"/>
+      <c r="L81" s="32" t="n"/>
+      <c r="M81" s="32" t="n"/>
+      <c r="N81" s="32" t="n"/>
+      <c r="O81" s="32" t="n"/>
+      <c r="P81" s="32" t="n"/>
+      <c r="Q81" s="32" t="n"/>
       <c r="R81" s="25" t="n"/>
       <c r="S81" s="25" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="29" t="inlineStr">
-        <is>
-          <t>Sharpe measures return relative to risk (volatility). A Sharpe of 1.5 means you're earning 1.5 units of return per unit of risk you're taking.</t>
-        </is>
-      </c>
-      <c r="B82" s="25" t="n"/>
-      <c r="C82" s="25" t="n"/>
-      <c r="D82" s="25" t="n"/>
-      <c r="E82" s="25" t="n"/>
-      <c r="F82" s="25" t="n"/>
-      <c r="G82" s="25" t="n"/>
-      <c r="H82" s="25" t="n"/>
-      <c r="I82" s="25" t="n"/>
-      <c r="J82" s="25" t="n"/>
-      <c r="K82" s="25" t="n"/>
-      <c r="L82" s="25" t="n"/>
-      <c r="M82" s="25" t="n"/>
-      <c r="N82" s="25" t="n"/>
-      <c r="O82" s="25" t="n"/>
-      <c r="P82" s="25" t="n"/>
-      <c r="Q82" s="25" t="n"/>
+      <c r="A82" s="44" t="n"/>
+      <c r="B82" s="32" t="n"/>
+      <c r="C82" s="32" t="n"/>
+      <c r="D82" s="32" t="n"/>
+      <c r="E82" s="32" t="n"/>
+      <c r="F82" s="32" t="n"/>
+      <c r="G82" s="32" t="n"/>
+      <c r="H82" s="32" t="n"/>
+      <c r="I82" s="32" t="n"/>
+      <c r="J82" s="32" t="n"/>
+      <c r="K82" s="32" t="n"/>
+      <c r="L82" s="32" t="n"/>
+      <c r="M82" s="32" t="n"/>
+      <c r="N82" s="32" t="n"/>
+      <c r="O82" s="32" t="n"/>
+      <c r="P82" s="32" t="n"/>
+      <c r="Q82" s="32" t="n"/>
       <c r="R82" s="25" t="n"/>
       <c r="S82" s="25" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="29" t="inlineStr">
-        <is>
-          <t>Above 1.0 is good; above 2.0 is great. It penalises strategies that are profitable but swing wildly — you want smooth, consistent gains.</t>
-        </is>
-      </c>
-      <c r="B83" s="25" t="n"/>
-      <c r="C83" s="25" t="n"/>
-      <c r="D83" s="25" t="n"/>
-      <c r="E83" s="25" t="n"/>
-      <c r="F83" s="25" t="n"/>
-      <c r="G83" s="25" t="n"/>
-      <c r="H83" s="25" t="n"/>
-      <c r="I83" s="25" t="n"/>
-      <c r="J83" s="25" t="n"/>
-      <c r="K83" s="25" t="n"/>
-      <c r="L83" s="25" t="n"/>
-      <c r="M83" s="25" t="n"/>
-      <c r="N83" s="25" t="n"/>
-      <c r="O83" s="25" t="n"/>
-      <c r="P83" s="25" t="n"/>
-      <c r="Q83" s="25" t="n"/>
+      <c r="A83" s="44" t="n"/>
+      <c r="B83" s="32" t="n"/>
+      <c r="C83" s="32" t="n"/>
+      <c r="D83" s="32" t="n"/>
+      <c r="E83" s="32" t="n"/>
+      <c r="F83" s="32" t="n"/>
+      <c r="G83" s="32" t="n"/>
+      <c r="H83" s="32" t="n"/>
+      <c r="I83" s="32" t="n"/>
+      <c r="J83" s="32" t="n"/>
+      <c r="K83" s="32" t="n"/>
+      <c r="L83" s="32" t="n"/>
+      <c r="M83" s="32" t="n"/>
+      <c r="N83" s="32" t="n"/>
+      <c r="O83" s="32" t="n"/>
+      <c r="P83" s="32" t="n"/>
+      <c r="Q83" s="32" t="n"/>
       <c r="R83" s="25" t="n"/>
       <c r="S83" s="25" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="25" t="n"/>
-      <c r="B84" s="25" t="n"/>
-      <c r="C84" s="25" t="n"/>
-      <c r="D84" s="25" t="n"/>
-      <c r="E84" s="25" t="n"/>
-      <c r="F84" s="25" t="n"/>
-      <c r="G84" s="25" t="n"/>
-      <c r="H84" s="25" t="n"/>
-      <c r="I84" s="25" t="n"/>
-      <c r="J84" s="25" t="n"/>
-      <c r="K84" s="25" t="n"/>
-      <c r="L84" s="25" t="n"/>
-      <c r="M84" s="25" t="n"/>
-      <c r="N84" s="25" t="n"/>
-      <c r="O84" s="25" t="n"/>
-      <c r="P84" s="25" t="n"/>
-      <c r="Q84" s="25" t="n"/>
+      <c r="A84" s="32" t="n"/>
+      <c r="B84" s="32" t="n"/>
+      <c r="C84" s="32" t="n"/>
+      <c r="D84" s="32" t="n"/>
+      <c r="E84" s="32" t="n"/>
+      <c r="F84" s="32" t="n"/>
+      <c r="G84" s="32" t="n"/>
+      <c r="H84" s="32" t="n"/>
+      <c r="I84" s="32" t="n"/>
+      <c r="J84" s="32" t="n"/>
+      <c r="K84" s="32" t="n"/>
+      <c r="L84" s="32" t="n"/>
+      <c r="M84" s="32" t="n"/>
+      <c r="N84" s="32" t="n"/>
+      <c r="O84" s="32" t="n"/>
+      <c r="P84" s="32" t="n"/>
+      <c r="Q84" s="32" t="n"/>
       <c r="R84" s="25" t="n"/>
       <c r="S84" s="25" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="25" t="inlineStr">
-        <is>
-          <t>Together</t>
-        </is>
-      </c>
-      <c r="B85" s="25" t="n"/>
-      <c r="C85" s="25" t="n"/>
-      <c r="D85" s="25" t="n"/>
-      <c r="E85" s="25" t="n"/>
-      <c r="F85" s="25" t="n"/>
-      <c r="G85" s="25" t="n"/>
-      <c r="H85" s="25" t="n"/>
-      <c r="I85" s="25" t="n"/>
-      <c r="J85" s="25" t="n"/>
-      <c r="K85" s="25" t="n"/>
-      <c r="L85" s="25" t="n"/>
-      <c r="M85" s="25" t="n"/>
-      <c r="N85" s="25" t="n"/>
-      <c r="O85" s="25" t="n"/>
-      <c r="P85" s="25" t="n"/>
-      <c r="Q85" s="25" t="n"/>
+      <c r="A85" s="32" t="n"/>
+      <c r="B85" s="32" t="n"/>
+      <c r="C85" s="32" t="n"/>
+      <c r="D85" s="32" t="n"/>
+      <c r="E85" s="32" t="n"/>
+      <c r="F85" s="32" t="n"/>
+      <c r="G85" s="32" t="n"/>
+      <c r="H85" s="32" t="n"/>
+      <c r="I85" s="32" t="n"/>
+      <c r="J85" s="32" t="n"/>
+      <c r="K85" s="32" t="n"/>
+      <c r="L85" s="32" t="n"/>
+      <c r="M85" s="32" t="n"/>
+      <c r="N85" s="32" t="n"/>
+      <c r="O85" s="32" t="n"/>
+      <c r="P85" s="32" t="n"/>
+      <c r="Q85" s="32" t="n"/>
       <c r="R85" s="25" t="n"/>
       <c r="S85" s="25" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="29" t="inlineStr">
-        <is>
-          <t>PF tells you "is this profitable?" and Sharpe tells you "is the ride smooth enough to actually hold through?"</t>
-        </is>
-      </c>
-      <c r="B86" s="25" t="n"/>
-      <c r="C86" s="25" t="n"/>
-      <c r="D86" s="25" t="n"/>
-      <c r="E86" s="25" t="n"/>
-      <c r="F86" s="25" t="n"/>
-      <c r="G86" s="25" t="n"/>
-      <c r="H86" s="25" t="n"/>
-      <c r="I86" s="25" t="n"/>
-      <c r="J86" s="25" t="n"/>
-      <c r="K86" s="25" t="n"/>
-      <c r="L86" s="25" t="n"/>
-      <c r="M86" s="25" t="n"/>
-      <c r="N86" s="25" t="n"/>
-      <c r="O86" s="25" t="n"/>
-      <c r="P86" s="25" t="n"/>
-      <c r="Q86" s="25" t="n"/>
+      <c r="A86" s="44" t="n"/>
+      <c r="B86" s="32" t="n"/>
+      <c r="C86" s="32" t="n"/>
+      <c r="D86" s="32" t="n"/>
+      <c r="E86" s="32" t="n"/>
+      <c r="F86" s="32" t="n"/>
+      <c r="G86" s="32" t="n"/>
+      <c r="H86" s="32" t="n"/>
+      <c r="I86" s="32" t="n"/>
+      <c r="J86" s="32" t="n"/>
+      <c r="K86" s="32" t="n"/>
+      <c r="L86" s="32" t="n"/>
+      <c r="M86" s="32" t="n"/>
+      <c r="N86" s="32" t="n"/>
+      <c r="O86" s="32" t="n"/>
+      <c r="P86" s="32" t="n"/>
+      <c r="Q86" s="32" t="n"/>
       <c r="R86" s="25" t="n"/>
       <c r="S86" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A6:Q6"/>
     <mergeCell ref="A58:Q58"/>
     <mergeCell ref="A39:Q39"/>
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="A6:Q6"/>
-    <mergeCell ref="A16:Q16"/>
-    <mergeCell ref="A25:Q25"/>
-    <mergeCell ref="A46:Q46"/>
     <mergeCell ref="A12:Q12"/>
     <mergeCell ref="A50:Q50"/>
+    <mergeCell ref="A16:Q16"/>
     <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A25:Q25"/>
     <mergeCell ref="A33:Q33"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A46:Q46"/>
     <mergeCell ref="A5:Q5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9491,7 +9470,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -9499,7 +9477,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
         <is>
@@ -9528,7 +9505,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
@@ -9536,7 +9512,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
@@ -9544,7 +9519,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="22" t="inlineStr">
         <is>
@@ -9559,7 +9533,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="22" t="inlineStr">
         <is>
@@ -9574,7 +9547,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="22" t="inlineStr">
         <is>
@@ -9589,7 +9561,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="22" t="inlineStr">
         <is>
@@ -9604,7 +9575,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="22" t="inlineStr">
         <is>
@@ -9619,7 +9589,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="22" t="inlineStr">
         <is>
@@ -9634,7 +9603,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="22" t="inlineStr">
         <is>
@@ -9649,7 +9617,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
@@ -9657,7 +9624,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="22" t="inlineStr">
         <is>
@@ -9679,7 +9645,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="22" t="inlineStr">
         <is>
@@ -9701,7 +9666,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
@@ -9709,7 +9673,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="B47" s="3" t="inlineStr">
         <is>
@@ -9800,8 +9763,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="19" t="inlineStr">
         <is>
@@ -9809,7 +9770,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="B55" s="3" t="inlineStr">
         <is>
@@ -10005,8 +9965,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
-    <row r="65"/>
     <row r="66">
       <c r="A66" s="19" t="inlineStr">
         <is>
@@ -10014,7 +9972,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="B68" s="3" t="inlineStr">
         <is>
@@ -10189,8 +10146,6 @@
         </is>
       </c>
     </row>
-    <row r="76"/>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="19" t="inlineStr">
         <is>
@@ -10198,7 +10153,6 @@
         </is>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="B80" s="3" t="inlineStr">
         <is>
@@ -10441,8 +10395,6 @@
         </is>
       </c>
     </row>
-    <row r="86"/>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="19" t="inlineStr">
         <is>
@@ -10450,7 +10402,6 @@
         </is>
       </c>
     </row>
-    <row r="89"/>
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
         <is>
@@ -10465,7 +10416,6 @@
         </is>
       </c>
     </row>
-    <row r="92"/>
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
         <is>
@@ -10480,7 +10430,6 @@
         </is>
       </c>
     </row>
-    <row r="95"/>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
@@ -10495,7 +10444,6 @@
         </is>
       </c>
     </row>
-    <row r="98"/>
     <row r="99">
       <c r="A99" s="14" t="inlineStr">
         <is>
@@ -10510,7 +10458,6 @@
         </is>
       </c>
     </row>
-    <row r="101"/>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
@@ -10525,7 +10472,6 @@
         </is>
       </c>
     </row>
-    <row r="104"/>
     <row r="105">
       <c r="A105" s="14" t="inlineStr">
         <is>
@@ -10540,7 +10486,6 @@
         </is>
       </c>
     </row>
-    <row r="107"/>
     <row r="108">
       <c r="A108" s="14" t="inlineStr">
         <is>
@@ -10555,8 +10500,6 @@
         </is>
       </c>
     </row>
-    <row r="110"/>
-    <row r="111"/>
     <row r="112">
       <c r="A112" s="23" t="inlineStr">
         <is>
@@ -10564,7 +10507,6 @@
         </is>
       </c>
     </row>
-    <row r="113"/>
     <row r="114">
       <c r="A114" s="21" t="inlineStr">
         <is>

</xml_diff>